<commit_message>
cập nhập nhập kho ( chỉnh sửa bảng liên kết )
</commit_message>
<xml_diff>
--- a/docs/System test (2).xlsx
+++ b/docs/System test (2).xlsx
@@ -20,9 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="38">
     <font>
@@ -370,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -719,6 +720,18 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="36" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1233,7 +1246,7 @@
           <t>Add information to Test Case</t>
         </is>
       </c>
-      <c r="F10" s="56" t="n"/>
+      <c r="F10" s="100" t="n"/>
     </row>
     <row r="11" ht="22.5" customHeight="1" s="103">
       <c r="A11" s="48" t="n">
@@ -1285,7 +1298,7 @@
           <t>Add test case User Account &amp; Role Configuration</t>
         </is>
       </c>
-      <c r="F12" s="56" t="n"/>
+      <c r="F12" s="100" t="n"/>
     </row>
     <row r="13" ht="22.5" customHeight="1" s="103">
       <c r="A13" s="48" t="n">
@@ -1337,7 +1350,7 @@
           <t>Add test case Point of Sale (POS) Order &amp; Payment</t>
         </is>
       </c>
-      <c r="F14" s="56" t="n"/>
+      <c r="F14" s="100" t="n"/>
     </row>
     <row r="15" ht="22.5" customHeight="1" s="103">
       <c r="A15" s="48" t="n">
@@ -1363,7 +1376,7 @@
           <t>Add test case Stocktaking &amp; Inventory Reconciliation</t>
         </is>
       </c>
-      <c r="F15" s="56" t="n"/>
+      <c r="F15" s="100" t="n"/>
     </row>
     <row r="16" ht="22.5" customHeight="1" s="103">
       <c r="A16" s="48" t="n">
@@ -1389,7 +1402,7 @@
           <t>Add test case Financial Cash Flow Recording</t>
         </is>
       </c>
-      <c r="F16" s="56" t="n"/>
+      <c r="F16" s="100" t="n"/>
     </row>
     <row r="17" ht="22.5" customHeight="1" s="103">
       <c r="A17" s="48" t="n">
@@ -1415,7 +1428,7 @@
           <t>Add test case Report Generation &amp; Business Analytics</t>
         </is>
       </c>
-      <c r="F17" s="56" t="n"/>
+      <c r="F17" s="100" t="n"/>
     </row>
     <row r="18" ht="22.5" customHeight="1" s="103">
       <c r="A18" s="75" t="n"/>
@@ -1423,14 +1436,14 @@
       <c r="C18" s="50" t="n"/>
       <c r="D18" s="76" t="n"/>
       <c r="E18" s="50" t="n"/>
-      <c r="F18" s="56" t="n"/>
+      <c r="F18" s="100" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B3:D3"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B3:D3"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B4:D4"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="A10:A18" showDropDown="1" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="custom">
@@ -1989,17 +2002,17 @@
         </is>
       </c>
       <c r="C12" s="41" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D12" s="41" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="41" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F12" s="41" t="n"/>
       <c r="G12" s="41" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -3308,7 +3321,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P43"/>
+  <dimension ref="B1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="19.5" customWidth="1" style="103" min="2" max="2"/>
@@ -4247,25 +4260,6 @@
     <row r="24">
       <c r="D24" s="97" t="n"/>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="C2:F2"/>
@@ -5694,7 +5688,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:P17"/>
+  <dimension ref="A1:P39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="19.13" customWidth="1" style="103" min="2" max="2"/>
@@ -5761,7 +5755,7 @@
         </is>
       </c>
       <c r="C3" s="117" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D3" s="105" t="n"/>
       <c r="E3" s="105" t="n"/>
@@ -5821,12 +5815,14 @@
         </is>
       </c>
       <c r="C5" s="39" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D5" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="39" t="n"/>
+      <c r="E5" s="39" t="n">
+        <v>0</v>
+      </c>
       <c r="F5" s="44" t="n">
         <v>0</v>
       </c>
@@ -5995,315 +5991,553 @@
           <t>Validate the creation of a receipt (quantity &gt; 0 &gt; 0), and the receipt approval process through the statuses "Pending Approval", "Rejected", and "Received".</t>
         </is>
       </c>
-      <c r="C10" s="105" t="n"/>
-      <c r="D10" s="105" t="n"/>
-      <c r="E10" s="105" t="n"/>
-      <c r="F10" s="105" t="n"/>
-      <c r="G10" s="105" t="n"/>
-      <c r="H10" s="105" t="n"/>
-      <c r="I10" s="105" t="n"/>
-      <c r="J10" s="105" t="n"/>
-      <c r="K10" s="105" t="n"/>
-      <c r="L10" s="105" t="n"/>
-      <c r="M10" s="105" t="n"/>
-      <c r="N10" s="105" t="n"/>
-      <c r="O10" s="105" t="n"/>
-      <c r="P10" s="106" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="80" t="inlineStr">
+      <c r="B11" s="131" t="inlineStr">
         <is>
           <t>SYS_INV_01</t>
         </is>
       </c>
-      <c r="C11" s="82" t="inlineStr">
-        <is>
-          <t>WarehouseStaff creates a Goods Import Order successfully</t>
-        </is>
-      </c>
-      <c r="D11" s="82" t="inlineStr">
+      <c r="C11" s="132" t="inlineStr">
+        <is>
+          <t>WarehouseStaff creates a Goods Import Order via Manual Entry mode (Pending Approval)</t>
+        </is>
+      </c>
+      <c r="D11" s="132" t="inlineStr">
         <is>
           <t>1. Log in as WarehouseStaff.
-2. Click the "Quản lý kho" menu and select the "Nhập hàng" tab to navigate to /inventory?tab=import.
-3. Click the "Tạo phiếu nhập" button.
-4. Fill in the import order details:
-- Nhà cung cấp: Select "Công ty TNHH Hải Nam"
-- Sản phẩm: Select "Sữa tươi Vinamilk 1L", Quantity: 100, Import price: 20,000đ
-- Ghi chú: Input "Nhập kho định kỳ tháng 7"
-5. Click the "Tạo phiếu" button.</t>
-        </is>
-      </c>
-      <c r="E11" s="82" t="inlineStr">
-        <is>
-          <t>- The system displays success message: "Tạo phiếu nhập hàng thành công và đang chờ duyệt."
-- The new import ticket appears in the list under the "Nhập hàng" tab with status "Chờ duyệt".</t>
-        </is>
-      </c>
-      <c r="F11" s="82" t="inlineStr">
-        <is>
-          <t>- An active WarehouseStaff account is logged in.
-- Supplier "Công ty TNHH Hải Nam" and product "Sữa tươi Vinamilk 1L" are pre-configured.</t>
-        </is>
-      </c>
-      <c r="G11" s="79" t="n"/>
-      <c r="H11" s="98" t="n">
-        <v>46224</v>
-      </c>
-      <c r="I11" s="84" t="n"/>
-      <c r="J11" s="79" t="n"/>
-      <c r="K11" s="84" t="n"/>
-      <c r="L11" s="84" t="n"/>
-      <c r="M11" s="79" t="n"/>
-      <c r="N11" s="84" t="n"/>
-      <c r="O11" s="84" t="n"/>
+2. Navigate to /inventory?tab=stock&amp;warehouseId=1.
+3. Click "Nhập Hàng" button to open modal #importStockModal.
+4. On tab "Nhập tay", type product name "Sữa tươi Vinamilk 1L" into search box #importSearchInput.
+5. Select matching product from dropdown. Select supplier "Công ty TNHH Hải Nam", enter import price 20000, and quantity 100.
+6. Enter optional note "Nhập kho định kỳ tháng 7".
+7. Click "Nhập hàng" button (#importSubmitBtn) to submit form (action=saveImport).</t>
+        </is>
+      </c>
+      <c r="E11" s="132" t="inlineStr">
+        <is>
+          <t>- System displays success message: "Đã tạo phiếu nhập hàng (Chờ duyệt)."
+- Purchase order is created in DB with status PENDING and code PO-[timestamp].
+- Physical inventory stock of "Sữa tươi Vinamilk 1L" is NOT updated yet.
+- No payment transaction is created in Cashbook yet.</t>
+        </is>
+      </c>
+      <c r="F11" s="132" t="inlineStr">
+        <is>
+          <t>- Active WarehouseStaff account is logged in.
+- Active warehouse is selected (selectedWarehouseId).
+- Products and active suppliers exist in system.</t>
+        </is>
+      </c>
+      <c r="G11" s="121" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H11" s="122" t="n">
+        <v>46228</v>
+      </c>
+      <c r="I11" s="123" t="inlineStr">
+        <is>
+          <t>ChiHTH</t>
+        </is>
+      </c>
+      <c r="J11" s="123" t="n"/>
+      <c r="K11" s="123" t="n"/>
+      <c r="L11" s="123" t="n"/>
+      <c r="M11" s="123" t="n"/>
+      <c r="N11" s="123" t="n"/>
+      <c r="O11" s="123" t="n"/>
       <c r="P11" s="84" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="80" t="inlineStr">
+      <c r="B12" s="131" t="inlineStr">
         <is>
           <t>SYS_INV_02</t>
         </is>
       </c>
-      <c r="C12" s="82" t="inlineStr">
-        <is>
-          <t>StoreManager approves the Goods Import Order and updates stock</t>
-        </is>
-      </c>
-      <c r="D12" s="82" t="inlineStr">
+      <c r="C12" s="132" t="inlineStr">
+        <is>
+          <t>StoreManager / Owner approves a pending Goods Import Order (Stock Increase &amp; Auto Cashbook Expense)</t>
+        </is>
+      </c>
+      <c r="D12" s="132" t="inlineStr">
         <is>
           <t>1. Log in as StoreManager.
-2. Click the "Quản lý kho" menu and select the "Chờ duyệt" tab at /inventory?tab=approval.
-3. Locate the pending import ticket from "Công ty TNHH Hải Nam" and click the "Xem chi tiết" button.
-4. Click the "Phê duyệt nhập kho" button.
-5. Fill out the received quantities and click the "Xác nhận nhận hàng" button on the receipt form.</t>
-        </is>
-      </c>
-      <c r="E12" s="82" t="inlineStr">
-        <is>
-          <t>- The system displays success message: "Phê duyệt phiếu nhập kho thành công. Hàng đã được nhập vào kho."
-- The ticket status updates to "Đã nhập kho".
-- The inventory stock count of "Sữa tươi Vinamilk 1L" increases by 100 units.</t>
-        </is>
-      </c>
-      <c r="F12" s="82" t="inlineStr">
-        <is>
-          <t>- A pending import ticket exists in the approval queue.
-- An active StoreManager account is logged in.</t>
-        </is>
-      </c>
-      <c r="G12" s="79" t="n"/>
-      <c r="H12" s="98" t="n">
-        <v>46224</v>
-      </c>
-      <c r="I12" s="84" t="n"/>
-      <c r="J12" s="79" t="n"/>
-      <c r="K12" s="84" t="n"/>
-      <c r="L12" s="84" t="n"/>
-      <c r="M12" s="79" t="n"/>
-      <c r="N12" s="84" t="n"/>
-      <c r="O12" s="84" t="n"/>
+2. Navigate to /inventory?tab=approval or /inventory?tab=history.
+3. Locate the pending purchase order and click "Xem chi tiết".
+4. Click "Duyệt phiếu" button (POST action=approveOrder&amp;orderId=... to /inventory-order).</t>
+        </is>
+      </c>
+      <c r="E12" s="132" t="inlineStr">
+        <is>
+          <t>- System displays success message: "Đã phê duyệt phiếu và cập nhật tồn kho thành công."
+- Order status in DB updates to COMPLETED.
+- Inventory stock count of "Sữa tươi Vinamilk 1L" increases directly by 100 units.
+- Stock transaction logged with type "IMPORT", source "PURCHASE_ORDER", notes "Nhập hàng từ phiếu PO-...".
+- An expense payment record (paymentType="EXPENSE", status="PAID") equal to order total amount is automatically created in Cashbook (payment table).</t>
+        </is>
+      </c>
+      <c r="F12" s="132" t="inlineStr">
+        <is>
+          <t>- Active StoreManager or Owner account is logged in.
+- A pending purchase order (PO-[timestamp], status PENDING) created by WarehouseStaff exists.</t>
+        </is>
+      </c>
+      <c r="G12" s="121" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H12" s="122" t="n">
+        <v>46228</v>
+      </c>
+      <c r="I12" s="123" t="inlineStr">
+        <is>
+          <t>ChiHTH</t>
+        </is>
+      </c>
+      <c r="J12" s="123" t="n"/>
+      <c r="K12" s="123" t="n"/>
+      <c r="L12" s="123" t="n"/>
+      <c r="M12" s="123" t="n"/>
+      <c r="N12" s="123" t="n"/>
+      <c r="O12" s="123" t="n"/>
       <c r="P12" s="84" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="118" t="inlineStr">
-        <is>
-          <t>The formula for adjusting inventory increases and recording the action log is in the "Inventory History" tab.</t>
-        </is>
-      </c>
-      <c r="C13" s="105" t="n"/>
-      <c r="D13" s="105" t="n"/>
-      <c r="E13" s="105" t="n"/>
-      <c r="F13" s="105" t="n"/>
-      <c r="G13" s="105" t="n"/>
-      <c r="H13" s="105" t="n"/>
-      <c r="I13" s="105" t="n"/>
-      <c r="J13" s="105" t="n"/>
-      <c r="K13" s="105" t="n"/>
-      <c r="L13" s="105" t="n"/>
-      <c r="M13" s="105" t="n"/>
-      <c r="N13" s="105" t="n"/>
-      <c r="O13" s="105" t="n"/>
-      <c r="P13" s="106" t="n"/>
+      <c r="B13" s="133" t="inlineStr">
+        <is>
+          <t>SYS_INV_03</t>
+        </is>
+      </c>
+      <c r="C13" s="125" t="inlineStr">
+        <is>
+          <t>StoreManager / Owner creates a Goods Import Order (Immediate Stock Increase &amp; Cashbook Expense)</t>
+        </is>
+      </c>
+      <c r="D13" s="125" t="inlineStr">
+        <is>
+          <t>1. Log in as StoreManager or Owner.
+2. Click "Nhập Hàng" button on /inventory?tab=stock.
+3. Search and add product "Sữa tươi Vinamilk 1L", select supplier, enter import price 20000 and quantity 50.
+4. Click "Nhập hàng" button.</t>
+        </is>
+      </c>
+      <c r="E13" s="125" t="inlineStr">
+        <is>
+          <t>- System displays success message: "Đã nhập hàng và cập nhật tồn kho thành công!"
+- Purchase order is created directly with status COMPLETED.
+- Inventory stock of "Sữa tươi Vinamilk 1L" increases immediately by 50 units.
+- Stock transaction logged as "IMPORT".
+- Expense payment record (EXPENSE, PAID) is automatically created in Cashbook.</t>
+        </is>
+      </c>
+      <c r="F13" s="125" t="inlineStr">
+        <is>
+          <t>- Active StoreManager or Owner account is logged in.
+- Active warehouse selected.</t>
+        </is>
+      </c>
+      <c r="G13" s="126" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H13" s="134" t="n">
+        <v>46228</v>
+      </c>
+      <c r="I13" s="127" t="inlineStr">
+        <is>
+          <t>ChiHTH</t>
+        </is>
+      </c>
+      <c r="J13" s="127" t="n"/>
+      <c r="K13" s="127" t="n"/>
+      <c r="L13" s="127" t="n"/>
+      <c r="M13" s="127" t="n"/>
+      <c r="N13" s="127" t="n"/>
+      <c r="O13" s="127" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="80" t="inlineStr">
-        <is>
-          <t>SYS_INV_03</t>
-        </is>
-      </c>
-      <c r="C14" s="82" t="inlineStr">
-        <is>
-          <t>StoreManager rejects the Goods Import Order</t>
-        </is>
-      </c>
-      <c r="D14" s="82" t="inlineStr">
+      <c r="B14" s="131" t="inlineStr">
+        <is>
+          <t>SYS_INV_04</t>
+        </is>
+      </c>
+      <c r="C14" s="132" t="inlineStr">
+        <is>
+          <t>WarehouseStaff imports goods using Excel file upload template (handleExcelUpload)</t>
+        </is>
+      </c>
+      <c r="D14" s="132" t="inlineStr">
+        <is>
+          <t>1. Log in as WarehouseStaff and click "Nhập Hàng" button on /inventory?tab=stock.
+2. Switch to tab "Nhập từ Excel".
+3. Click "Tải file mẫu" (downloadExcelTemplate()) to get .xlsx template.
+4. Fill template Excel with columns: Tên sản phẩm ("Sữa tươi Vinamilk 1L"), Mã NCC (1), Tên NCC, Số lượng nhập (100). Save file.
+5. On modal, click "Chọn file Excel" (handleExcelUpload()) and select the .xlsx file.
+6. JS parses file, matches products, populates #excelImportProductTableBody, and enables "Nhập hàng" button.
+7. Click "Nhập hàng" button.</t>
+        </is>
+      </c>
+      <c r="E14" s="132" t="inlineStr">
+        <is>
+          <t>- System displays success message: "Đã tạo phiếu nhập hàng (Chờ duyệt)."
+- Import order created with status PENDING.</t>
+        </is>
+      </c>
+      <c r="F14" s="132" t="inlineStr">
+        <is>
+          <t>- Active WarehouseStaff account is logged in.
+- Downloaded Excel import template Mau_Nhap_Hang_[Date].xlsx.</t>
+        </is>
+      </c>
+      <c r="G14" s="121" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H14" s="122" t="n">
+        <v>46228</v>
+      </c>
+      <c r="I14" s="123" t="inlineStr">
+        <is>
+          <t>ChiHTH</t>
+        </is>
+      </c>
+      <c r="J14" s="123" t="n"/>
+      <c r="K14" s="123" t="n"/>
+      <c r="L14" s="123" t="n"/>
+      <c r="M14" s="123" t="n"/>
+      <c r="N14" s="123" t="n"/>
+      <c r="O14" s="123" t="n"/>
+      <c r="P14" s="84" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="131" t="inlineStr">
+        <is>
+          <t>SYS_INV_05</t>
+        </is>
+      </c>
+      <c r="C15" s="132" t="inlineStr">
+        <is>
+          <t>StoreManager rejects a pending Goods Import Order (rejectOrder)</t>
+        </is>
+      </c>
+      <c r="D15" s="132" t="inlineStr">
         <is>
           <t>1. Log in as StoreManager.
-2. Navigate to the "Chờ duyệt" tab under "Quản lý kho".
-3. Locate the target pending import ticket and click the "Từ chối" button.
-4. Input the rejection reason: "Sai thông tin đơn giá nhập" in the dialog box.
-5. Click the "Xác nhận từ chối" button.</t>
-        </is>
-      </c>
-      <c r="E14" s="82" t="inlineStr">
-        <is>
-          <t>- The system displays success message: "Từ chối phiếu nhập thành công."
-- The ticket status updates to "Bị từ chối" (Rejected).
-- The physical inventory stock is not modified.</t>
-        </is>
-      </c>
-      <c r="F14" s="82" t="inlineStr">
-        <is>
-          <t>- A pending import ticket exists in the approval queue.</t>
-        </is>
-      </c>
-      <c r="G14" s="79" t="n"/>
-      <c r="H14" s="98" t="n">
-        <v>46224</v>
-      </c>
-      <c r="I14" s="84" t="n"/>
-      <c r="J14" s="79" t="n"/>
-      <c r="K14" s="84" t="n"/>
-      <c r="L14" s="84" t="n"/>
-      <c r="M14" s="79" t="n"/>
-      <c r="N14" s="84" t="n"/>
-      <c r="O14" s="84" t="n"/>
-      <c r="P14" s="84" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="80" t="inlineStr">
-        <is>
-          <t>SYS_INV_04</t>
-        </is>
-      </c>
-      <c r="C15" s="82" t="inlineStr">
-        <is>
-          <t>WarehouseStaff attempts to create an import order with invalid quantity</t>
-        </is>
-      </c>
-      <c r="D15" s="82" t="inlineStr">
-        <is>
-          <t>1. Navigate to /inventory?tab=import as WarehouseStaff.
-2. Click "Tạo phiếu nhập".
-3. Fill in the supplier, select product "Sữa tươi Vinamilk 1L", and input a negative quantity: "-50".
-4. Click "Tạo phiếu".</t>
-        </is>
-      </c>
-      <c r="E15" s="82" t="inlineStr">
-        <is>
-          <t>- The form submission is blocked.
-- The system displays validation error: "Số lượng nhập phải lớn hơn 0."</t>
-        </is>
-      </c>
-      <c r="F15" s="82" t="inlineStr">
-        <is>
-          <t>- WarehouseStaff is logged in.</t>
-        </is>
-      </c>
-      <c r="G15" s="79" t="n"/>
-      <c r="H15" s="98" t="n">
-        <v>46224</v>
-      </c>
-      <c r="I15" s="84" t="n"/>
-      <c r="J15" s="79" t="n"/>
-      <c r="K15" s="84" t="n"/>
-      <c r="L15" s="84" t="n"/>
-      <c r="M15" s="79" t="n"/>
-      <c r="N15" s="84" t="n"/>
-      <c r="O15" s="84" t="n"/>
+2. Navigate to /inventory?tab=approval or /inventory?tab=history.
+3. Locate target pending import order and click "Từ chối" button.</t>
+        </is>
+      </c>
+      <c r="E15" s="132" t="inlineStr">
+        <is>
+          <t>- System displays success message: "Đã từ chối phiếu."
+- Order status in DB updates to REJECTED.
+- Physical inventory stock is NOT modified.
+- No Cashbook expense record is created.</t>
+        </is>
+      </c>
+      <c r="F15" s="132" t="inlineStr">
+        <is>
+          <t>- Active StoreManager account is logged in.
+- A pending purchase order (PENDING) exists in approval queue.</t>
+        </is>
+      </c>
+      <c r="G15" s="121" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H15" s="122" t="n">
+        <v>46228</v>
+      </c>
+      <c r="I15" s="123" t="inlineStr">
+        <is>
+          <t>ChiHTH</t>
+        </is>
+      </c>
+      <c r="J15" s="123" t="n"/>
+      <c r="K15" s="123" t="n"/>
+      <c r="L15" s="123" t="n"/>
+      <c r="M15" s="123" t="n"/>
+      <c r="N15" s="123" t="n"/>
+      <c r="O15" s="123" t="n"/>
       <c r="P15" s="84" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="80" t="inlineStr">
-        <is>
-          <t>SYS_INV_05</t>
-        </is>
-      </c>
-      <c r="C16" s="82" t="inlineStr">
-        <is>
-          <t>WarehouseStaff views the Inventory History tab to verify stock changes</t>
-        </is>
-      </c>
-      <c r="D16" s="82" t="inlineStr">
-        <is>
-          <t>1. Navigate to /inventory as WarehouseStaff.
-2. Click on the "Lịch sử kho" tab at /inventory?tab=history.</t>
-        </is>
-      </c>
-      <c r="E16" s="82" t="inlineStr">
-        <is>
-          <t>- The system loads a paginated history list of all stock changes.
-- The recent import of "100 units of Sữa tươi Vinamilk 1L" is listed, showing transaction type "Nhập hàng", and the modified timestamp matches the approval event.</t>
-        </is>
-      </c>
-      <c r="F16" s="82" t="inlineStr">
-        <is>
-          <t>- An import ticket was approved and completed previously.</t>
-        </is>
-      </c>
-      <c r="G16" s="101" t="n"/>
-      <c r="H16" s="98" t="n">
-        <v>46224</v>
-      </c>
-      <c r="I16" s="101" t="n"/>
-      <c r="J16" s="101" t="n"/>
-      <c r="K16" s="101" t="n"/>
-      <c r="L16" s="101" t="n"/>
-      <c r="M16" s="101" t="n"/>
-      <c r="N16" s="101" t="n"/>
-      <c r="O16" s="101" t="n"/>
+      <c r="B16" s="131" t="inlineStr">
+        <is>
+          <t>SYS_INV_06</t>
+        </is>
+      </c>
+      <c r="C16" s="132" t="inlineStr">
+        <is>
+          <t>WarehouseStaff cancels a pending Goods Import Order created by themselves (cancelOrder)</t>
+        </is>
+      </c>
+      <c r="D16" s="132" t="inlineStr">
+        <is>
+          <t>1. Log in as the WarehouseStaff creator.
+2. Navigate to /inventory?tab=pending_vouchers or /inventory?tab=stock.
+3. Locate the pending purchase order and click "Hủy phiếu" button.</t>
+        </is>
+      </c>
+      <c r="E16" s="132" t="inlineStr">
+        <is>
+          <t>- System displays success message: "Đã hủy phiếu thành công."
+- Order status in DB updates to CANCELLED.
+- Physical stock is NOT modified.</t>
+        </is>
+      </c>
+      <c r="F16" s="132" t="inlineStr">
+        <is>
+          <t>- Active WarehouseStaff account is logged in.
+- A pending purchase order (PENDING) created by this WarehouseStaff exists.</t>
+        </is>
+      </c>
+      <c r="G16" s="126" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H16" s="122" t="n">
+        <v>46228</v>
+      </c>
+      <c r="I16" s="127" t="inlineStr">
+        <is>
+          <t>ChiHTH</t>
+        </is>
+      </c>
+      <c r="J16" s="127" t="n"/>
+      <c r="K16" s="127" t="n"/>
+      <c r="L16" s="127" t="n"/>
+      <c r="M16" s="127" t="n"/>
+      <c r="N16" s="127" t="n"/>
+      <c r="O16" s="127" t="n"/>
       <c r="P16" s="101" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="80" t="inlineStr">
-        <is>
-          <t>SYS_INV_06</t>
-        </is>
-      </c>
-      <c r="C17" s="82" t="inlineStr">
-        <is>
-          <t>StoreManager approves warehouse transfer dispatch</t>
-        </is>
-      </c>
-      <c r="D17" s="82" t="inlineStr">
-        <is>
-          <t>1. Log in as StoreManager.
-2. Navigate to the "Duyệt yêu cầu" list at /inventory?tab=approval.
-3. Select a pending warehouse transfer request ticket (Stock Transfer).
-4. Click "Duyệt chuyển kho".</t>
-        </is>
-      </c>
-      <c r="E17" s="82" t="inlineStr">
-        <is>
-          <t>- The system displays success message: "Đã phê duyệt lệnh điều chuyển kho."
-- The source warehouse stock decreases, and the destination warehouse stock shows the inbound pending status.</t>
-        </is>
-      </c>
-      <c r="F17" s="82" t="inlineStr">
-        <is>
-          <t>- A stock transfer request was initiated between two warehouses.</t>
-        </is>
-      </c>
-      <c r="G17" s="101" t="n"/>
-      <c r="H17" s="98" t="n">
-        <v>46224</v>
-      </c>
-      <c r="I17" s="101" t="n"/>
-      <c r="J17" s="101" t="n"/>
-      <c r="K17" s="101" t="n"/>
-      <c r="L17" s="101" t="n"/>
-      <c r="M17" s="101" t="n"/>
-      <c r="N17" s="101" t="n"/>
-      <c r="O17" s="101" t="n"/>
+      <c r="B17" s="131" t="inlineStr">
+        <is>
+          <t>SYS_INV_07</t>
+        </is>
+      </c>
+      <c r="C17" s="132" t="inlineStr">
+        <is>
+          <t>WarehouseStaff attempts to approve a Goods Import Order (Permission Denial)</t>
+        </is>
+      </c>
+      <c r="D17" s="132" t="inlineStr">
+        <is>
+          <t>1. Log in as WarehouseStaff.
+2. Attempt to send HTTP POST request to /inventory-order with action=approveOrder&amp;orderId=123.</t>
+        </is>
+      </c>
+      <c r="E17" s="132" t="inlineStr">
+        <is>
+          <t>- Server blocks request and returns HTTP 403 Forbidden.
+- WarehouseStaff cannot approve purchase orders.</t>
+        </is>
+      </c>
+      <c r="F17" s="132" t="inlineStr">
+        <is>
+          <t>- Active WarehouseStaff account is logged in.
+- A pending purchase order exists.</t>
+        </is>
+      </c>
+      <c r="G17" s="126" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H17" s="122" t="n">
+        <v>46228</v>
+      </c>
+      <c r="I17" s="127" t="inlineStr">
+        <is>
+          <t>ChiHTH</t>
+        </is>
+      </c>
+      <c r="J17" s="127" t="n"/>
+      <c r="K17" s="127" t="n"/>
+      <c r="L17" s="127" t="n"/>
+      <c r="M17" s="127" t="n"/>
+      <c r="N17" s="127" t="n"/>
+      <c r="O17" s="127" t="n"/>
       <c r="P17" s="101" t="n"/>
     </row>
+    <row r="18">
+      <c r="B18" s="124" t="inlineStr">
+        <is>
+          <t>SYS_INV_08</t>
+        </is>
+      </c>
+      <c r="C18" s="125" t="inlineStr">
+        <is>
+          <t>WarehouseStaff attempts to create a Goods Import Order with invalid quantity (qty &lt;= 0)</t>
+        </is>
+      </c>
+      <c r="D18" s="125" t="inlineStr">
+        <is>
+          <t>1. Log in as WarehouseStaff and open #importStockModal.
+2. Select product, select supplier, enter quantity 0 (or -5).
+3. Send form submission.</t>
+        </is>
+      </c>
+      <c r="E18" s="125" t="inlineStr">
+        <is>
+          <t>- Submission is blocked by validation.
+- System displays error message: "Dòng 1: Số lượng nhập phải là số nguyên dương lớn hơn 0."</t>
+        </is>
+      </c>
+      <c r="F18" s="125" t="inlineStr">
+        <is>
+          <t>- Active WarehouseStaff account is logged in.</t>
+        </is>
+      </c>
+      <c r="G18" s="126" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H18" s="134" t="n">
+        <v>46228</v>
+      </c>
+      <c r="I18" s="127" t="inlineStr">
+        <is>
+          <t>ChiHTH</t>
+        </is>
+      </c>
+      <c r="J18" s="127" t="n"/>
+      <c r="K18" s="127" t="n"/>
+      <c r="L18" s="127" t="n"/>
+      <c r="M18" s="127" t="n"/>
+      <c r="N18" s="127" t="n"/>
+      <c r="O18" s="127" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="124" t="inlineStr">
+        <is>
+          <t>SYS_INV_09</t>
+        </is>
+      </c>
+      <c r="C19" s="125" t="inlineStr">
+        <is>
+          <t>WarehouseStaff attempts to create a Goods Import Order with duplicate product IDs</t>
+        </is>
+      </c>
+      <c r="D19" s="125" t="inlineStr">
+        <is>
+          <t>1. Log in as WarehouseStaff and open #importStockModal.
+2. Add product "Sữa tươi Vinamilk 1L" twice as separate rows in the same import form.
+3. Click "Nhập hàng" button.</t>
+        </is>
+      </c>
+      <c r="E19" s="125" t="inlineStr">
+        <is>
+          <t>- Submission is blocked by backend validation.
+- System displays error message: "Dòng 2: Sản phẩm ID [pId] bị lặp lại trong phiếu nhập."</t>
+        </is>
+      </c>
+      <c r="F19" s="125" t="inlineStr">
+        <is>
+          <t>- Active WarehouseStaff account is logged in.</t>
+        </is>
+      </c>
+      <c r="G19" s="126" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H19" s="134" t="n">
+        <v>46228</v>
+      </c>
+      <c r="I19" s="127" t="inlineStr">
+        <is>
+          <t>ChiHTH</t>
+        </is>
+      </c>
+      <c r="J19" s="127" t="n"/>
+      <c r="K19" s="127" t="n"/>
+      <c r="L19" s="127" t="n"/>
+      <c r="M19" s="127" t="n"/>
+      <c r="N19" s="127" t="n"/>
+      <c r="O19" s="127" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="124" t="inlineStr">
+        <is>
+          <t>SYS_INV_10</t>
+        </is>
+      </c>
+      <c r="C20" s="125" t="inlineStr">
+        <is>
+          <t>WarehouseStaff searches products available for import via API (searchImportProductsApi)</t>
+        </is>
+      </c>
+      <c r="D20" s="125" t="inlineStr">
+        <is>
+          <t>1. Send GET request to /inventory?action=searchImportProductsApi&amp;keyword=Vinamilk&amp;warehouseId=1.</t>
+        </is>
+      </c>
+      <c r="E20" s="125" t="inlineStr">
+        <is>
+          <t>- System returns HTTP 200 OK with JSON array of matching products containing productId, productName, productCodebar, categoryName, importPrice, supplierId, and supplierName.</t>
+        </is>
+      </c>
+      <c r="F20" s="125" t="inlineStr">
+        <is>
+          <t>- WarehouseStaff is logged in.
+- Product and supplier records exist.</t>
+        </is>
+      </c>
+      <c r="G20" s="126" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H20" s="134" t="n">
+        <v>46228</v>
+      </c>
+      <c r="I20" s="127" t="inlineStr">
+        <is>
+          <t>ChiHTH</t>
+        </is>
+      </c>
+      <c r="J20" s="127" t="n"/>
+      <c r="K20" s="127" t="n"/>
+      <c r="L20" s="127" t="n"/>
+      <c r="M20" s="127" t="n"/>
+      <c r="N20" s="127" t="n"/>
+      <c r="O20" s="127" t="n"/>
+    </row>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="3">
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="C1:F1"/>
     <mergeCell ref="C3:F3"/>
-    <mergeCell ref="B10:P10"/>
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="B13:P13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>